<commit_message>
docs: mark day one complete
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -83,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -93,6 +93,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -737,14 +740,22 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>GitHub governance, public GHCR, Entra OIDC/RBAC, and local five-container flow completed. Fixed missing nginx /api proxy. Containers and pgdata volume destroyed.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2181,7 +2192,7 @@
     <dataValidation sqref="J2:J28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Done,Skipped"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="L2:L28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,-"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3248,15 +3259,19 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>keep (local)</t>
+          <t>destroyed after verification</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>docs/LEARNING_JOURNAL.md#day-1--github-governance-azure-oidc-and-first-local-run</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -3597,6 +3612,39 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>local (no Azure RG)</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>GitHub/Entra setup + Docker Compose</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" s="7" t="inlineStr">
+        <is>
+          <t>Local stack and pgdata volume removed; reusable $0 identity/config retained</t>
+        </is>
+      </c>
+    </row>
     <row r="40">
       <c r="D40" s="5" t="inlineStr">
         <is>
@@ -3630,56 +3678,56 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Run at the END of EVERY session. No exceptions.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>1. SCREENSHOT dashboards first (portfolio evidence)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>2. az group list -o table   -- know exactly what exists</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>3. az group delete -n learn-&lt;stage&gt;-&lt;date&gt; --yes --no-wait</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>4. Terraform days: cd infra/&lt;day&gt; &amp;&amp; terraform destroy  -- review: must list only today's resources</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>5. az resource list -o table | grep &lt;date&gt;   -- no orphaned disks/NICs/IPs</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>6. az consumption usage list --top 5 -o table   -- know today's cost</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>7. Next morning: az group list   -- nothing unexpected alive</t>
         </is>

</xml_diff>

<commit_message>
docs: explain day two Azure foundations
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -803,14 +803,18 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Company-managed Windows laptop requires an IT administrator for Azure CLI installation. Use ephemeral Azure Cloud Shell; no resource has been created yet.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">

</xml_diff>

<commit_message>
docs: accelerate plan for GenAI sprint
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -8,11 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Daily Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Day Cost Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Deployments" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Cost Log" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Destroy Ritual" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="GenAI Sprint" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Daily Plan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Day Cost Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Deployments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cost Log" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Destroy Ritual" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,10 +49,10 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -91,8 +92,8 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -481,120 +482,120 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>App</t>
+          <t>Active app</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Feedback Analyzer (FastAPI + Celery + React) - one app, many deployments</t>
+          <t>Minimal synchronous FastAPI GenAI API - deployment depth over app complexity</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Window</t>
+          <t>Active window</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Aug 31 - Sep 27 2026, ~1 h/day (Day 22 AKS = 2 h)</t>
+          <t>Sep 26-27 2026, 16-hour accelerated sprint; destroy by Sep 27 20:00 IST</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Budget</t>
+          <t>Credit evidence</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>$200 trial credit; planned spend ~$8-15 (see Day Cost Plan); destroy same-day</t>
+          <t>INR 19,109.25 remaining; portal displays Sep 28 expiry; do not rely on Sep 28</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Golden rule</t>
+          <t>Sprint budget</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>A day is Done only when Destroyed? = Yes (except keep-listed items)</t>
+          <t>Expected &lt;INR 500; hard cap INR 1,500; see 'GenAI Sprint' tab</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Your role</t>
+          <t>Golden rule</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Portal clicks, az commands, terraform plan review + apply, verification</t>
+          <t>A day is Done only when Destroyed? = Yes (except keep-listed items)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Agent's job</t>
+          <t>Your role</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>TF files + exact commands prepared before each session; docs updated</t>
+          <t>Portal clicks, az commands, terraform plan review + apply, verification</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Docs</t>
+          <t>Agent's job</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>docs/LEARNING_PLAN.md · docs/DAILY_PLAYBOOK.md · docs/RUNBOOK.md</t>
+          <t>TF files + exact commands prepared before each session; docs updated</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Website deployment</t>
+          <t>Docs</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Day 19 (Sat Sep 19): React UI on Azure Static Web Apps, its own URL</t>
+          <t>docs/LEARNING_PLAN.md · docs/DAILY_PLAYBOOK.md · docs/RUNBOOK.md</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Deployments target</t>
+          <t>Paused curriculum</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>10 tracked deployments — see 'Deployments' tab</t>
+          <t>The original 28-day plan remains for later; VM, AKS, database, and frontend stages are paused</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Cost tab</t>
+          <t>Cost tabs</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>'Day Cost Plan' = planned cost per day + cumulative; 'Cost Log' = what you actually spent</t>
+          <t>'GenAI Sprint' tracks the active blocks; legacy Day Cost Plan is retained; Cost Log records actuals</t>
         </is>
       </c>
     </row>
@@ -604,6 +605,616 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Sprint day</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Azure services</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Cost guardrail</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Destroyed?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Expiry, budget, subscription, quotas, providers</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Cost Management, Resource Providers</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>₹0</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Architecture + tagged disposable resource group</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Resource Group, RBAC, tags</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>₹0</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Create Foundry resource and project manually</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Foundry</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>usage-based</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Deploy/test a small pay-as-you-go chat model</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Foundry Models</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹100 target</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Minimal synchronous FastAPI /health + /chat</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Local Python/Docker</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>₹0</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Build, tag, and push private image</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ACR Basic</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹30 target</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Deploy HTTPS scale-to-zero API with telemetry</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Container Apps, Log Analytics, App Insights</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹100 target</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Day A</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Managed identity, least privilege, Key Vault</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Entra ID, RBAC, Key Vault</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹20 target</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Upload two safe grounding documents</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Blob Storage Standard LRS</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹10 target</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Create search service/index and lexical retrieval</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Azure AI Search</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Free preferred</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Embeddings, vector retrieval, grounded RAG</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>AI Search + Foundry embedding/chat models</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹100 target</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Import OpenAPI and add rate limiting</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>APIM Consumption</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>near ₹0</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Content filters, prompt injection, mini evaluation</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Foundry safety/evaluation</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹100 target</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>OIDC build/publish/deploy immutable revision</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>GitHub Actions, ACR, Container Apps</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹50 target</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Logs, tiny load test, alert, revision rollback</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Azure Monitor, Container Apps revisions</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>&lt;₹100 target</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Day B</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Evidence, actual cost, delete and prove absence</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Cost Management, Resource Group</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>₹0</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Delete sprint RG and verify absence by Sep 27 20:00 IST</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Hard cap</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>INR 1,500; stop before any unexpected paid tier</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="F2:F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not started,In progress,Done,Skipped,Blocked"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No,-"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -812,7 +1423,7 @@
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Company-managed Windows laptop requires an IT administrator for Azure CLI installation. Use ephemeral Azure Cloud Shell; no resource has been created yet.</t>
+          <t>Accelerated two-day GenAI sprint started after portal confirmed INR 19,109.25 credit expires Sep 28. Use ephemeral Cloud Shell; destroy by Sep 27 20:00 IST.</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2815,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3187,7 +3798,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3561,7 +4172,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3669,7 +4280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: map Azure free quotas to GenAI sprint
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="GenAI Sprint" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Daily Plan" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Day Cost Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Deployments" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cost Log" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Destroy Ritual" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Free Quotas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Daily Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Day Cost Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Deployments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cost Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Destroy Ritual" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -841,12 +842,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ACR Basic</t>
+          <t>ACR Standard (12-month grant)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹30 target</t>
+          <t>free-quota target</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -1215,6 +1216,564 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Included amount</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Sprint decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>AI/RAG</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Azure AI Search</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>50 MB; 10,000 documents; 3 indexes</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Core: Free SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Hosting</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Container Apps Consumption</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>180,000 vCPU-s; 360,000 GiB-s; 2M requests/month</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Core: scale to zero</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Gateway</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>API Management Consumption</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Monthly included</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>First 1M API operations/subscription/month</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Content Safety F0</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Free tier</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>5,000 text records + 5,000 images/month; hard stop</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Registry</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Container Registry Standard</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>1 registry; 100 GB; 10 webhooks</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Core: exact Standard SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Blob Storage Hot LRS</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>5 GB; 20,000 reads; 10,000 writes</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Key Vault Standard</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>10,000 RSA-2048 key or secret operations</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Document AI</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Document Intelligence S0</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>500 pages</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>NLP</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Azure Language</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>5,000 text records</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Stretch</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Functions Consumption</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Monthly grant</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1M executions + 400,000 GB-s</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Stretch ingestion</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Event Grid</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>100,000 operations/month</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Stretch Blob trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Messaging</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Service Bus Standard</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>750 hours + 13M operations</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Defer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Cosmos DB free tier</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>1,000 RU/s + 25 GB when free tier selected</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Defer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>PostgreSQL Flexible B1ms</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>750 hours + 32 GB data + 32 GB backup</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Defer</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Compute</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Eligible Linux/Windows VMs</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>12 months</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>750 hours each for listed B1s/B2pts v2/B2ats v2</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Defer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AI platform</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Foundry</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Platform free</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Consumed features bill at their own rates</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Foundry/OpenAI inference</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>No general free-token grant; model/token rates</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Core: strict limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Observability</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Azure Monitor / Log Analytics</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Paid ingestion</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Platform metrics/activity logs have free units; log ingestion metered</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Core: sample/cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Important</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Quotas reset monthly and do not roll over. Exact SKU and the subscription's Cost Management &gt; Free services grid are authoritative. PAYG overages bill the card.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Official list</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://azure.microsoft.com/en-us/pricing/free-services/</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2632,7 +3191,7 @@
         </is>
       </c>
       <c r="K25" s="2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="L25" s="2" t="inlineStr"/>
       <c r="M25" s="2" t="inlineStr"/>
@@ -2815,7 +3374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3660,23 +4219,23 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>first 5GB ingestion/month free</t>
+          <t>log ingestion metered; platform metrics free</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>MBs</t>
+          <t>tiny</t>
         </is>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>7.8</v>
+        <v>7.85</v>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>First 5GB ingestion/month free</t>
+          <t>Log ingestion is metered; keep volume tiny</t>
         </is>
       </c>
     </row>
@@ -3708,7 +4267,7 @@
         <v>0.05</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>7.85</v>
+        <v>7.9</v>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
     </row>
@@ -3740,7 +4299,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>7.85</v>
+        <v>7.9</v>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
     </row>
@@ -3772,7 +4331,7 @@
         <v>0.41</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>8.26</v>
+        <v>8.31</v>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
     </row>
@@ -3783,7 +4342,7 @@
         </is>
       </c>
       <c r="G29" s="6" t="n">
-        <v>8.26</v>
+        <v>8.31</v>
       </c>
     </row>
     <row r="30">
@@ -3798,7 +4357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4172,7 +4731,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4280,7 +4839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: plan three Azure GenAI deployments
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Active app</t>
+          <t>Active apps</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Minimal synchronous FastAPI GenAI API - deployment depth over app complexity</t>
+          <t>One shared React SPA + three small FastAPI APIs: Chat, Document Q&amp;A, approval-gated Agent</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>docs/LEARNING_PLAN.md · docs/DAILY_PLAYBOOK.md · docs/RUNBOOK.md</t>
+          <t>1) GENAI_SOLUTION_OVERVIEW.md/html · 2) GENAI_DEPLOYMENT_GUIDE.md/html · 3) LEARNING_JOURNAL.md/html</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>The original 28-day plan remains for later; VM, AKS, database, and frontend stages are paused</t>
+          <t>The original 28-day plan remains for later; VM and AKS stages are paused</t>
         </is>
       </c>
     </row>
@@ -709,17 +709,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Architecture + tagged disposable resource group</t>
+          <t>Three flows + local shared React SPA and FastAPI contracts + shared cloud platform</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Resource Group, RBAC, tags</t>
+          <t>React, FastAPI, RG, Foundry, ACR, Key Vault, Monitor</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>₹0</t>
+          <t>&lt;₹100 target</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -741,17 +741,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Create Foundry resource and project manually</t>
+          <t>App 1 FastAPI on Fargate-equivalent hosting + React Chat page</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Foundry</t>
+          <t>Container Apps, Static Web Apps, ACR</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>usage-based</t>
+          <t>free-quota target</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -773,17 +773,17 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Deploy/test a small pay-as-you-go chat model</t>
+          <t>Cache MISS→HIT, managed identity, APIM, trusted HTTPS certificate</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Foundry Models</t>
+          <t>Azure Managed Redis, RBAC, APIM</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹100 target</t>
+          <t>Redis estimate required</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -805,17 +805,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Minimal synchronous FastAPI /health + /chat</t>
+          <t>Concurrent users, autoscaling, stampede lock, break/fix, revision rollback</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Local Python/Docker</t>
+          <t>Container Apps, Redis, App Insights</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>₹0</t>
+          <t>&lt;₹100 target</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -837,17 +837,17 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Build, tag, and push private image</t>
+          <t>Repeat App 1 deployment from learner's saved commands</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ACR Standard (12-month grant)</t>
+          <t>ACR, Container Apps, APIM</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>free-quota target</t>
+          <t>&lt;₹50 target</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -869,12 +869,12 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Deploy HTTPS scale-to-zero API with telemetry</t>
+          <t>Blob, AI Search, Content Safety, lexical/vector retrieval</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Container Apps, Log Analytics, App Insights</t>
+          <t>Storage, AI Search Free, Content Safety F0</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -901,17 +901,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Managed identity, least privilege, Key Vault</t>
+          <t>App 2 FastAPI + React Document Q&amp;A; grounded and unknown answers</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Entra ID, RBAC, Key Vault</t>
+          <t>Container Apps, Static Web Apps, Foundry, AI Search</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹20 target</t>
+          <t>&lt;₹100 target</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Upload two safe grounding documents</t>
+          <t>Durable runtime, queue TTL/dead letter, Cosmos item TTL</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Blob Storage Standard LRS</t>
+          <t>Functions, Storage, Service Bus, Cosmos DB</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹10 target</t>
+          <t>free-quota target</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -965,17 +965,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Create search service/index and lexical retrieval</t>
+          <t>App 3 FastAPI + React Agent page + approval orchestrator + worker</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Azure AI Search</t>
+          <t>Container Apps, Static Web Apps, Durable Functions</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Free preferred</t>
+          <t>&lt;₹100 target</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -997,17 +997,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Embeddings, vector retrieval, grounded RAG</t>
+          <t>Concurrent runs: approve, reject, approval timeout, queue depth</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>AI Search + Foundry embedding/chat models</t>
+          <t>Durable Functions, Service Bus, Cosmos DB</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹100 target</t>
+          <t>&lt;₹50 target</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1029,17 +1029,17 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Import OpenAPI and add rate limiting</t>
+          <t>Duplicate/changed approval, message expiry, retry, dead letter, replay, lock renewal</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>APIM Consumption</t>
+          <t>Service Bus, Durable Functions, App Insights</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>near ₹0</t>
+          <t>&lt;₹50 target</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1061,17 +1061,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Content filters, prompt injection, mini evaluation</t>
+          <t>Three APIM routes, HTTPS-only, certificate inspection, rate limits</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Foundry safety/evaluation</t>
+          <t>APIM Consumption, managed TLS</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>&lt;₹100 target</t>
+          <t>near ₹0</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Logs, tiny load test, alert, revision rollback</t>
+          <t>Cross-app logs, tiny load tests, alert, independent repeat deployment</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1315,49 +1315,49 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Gateway</t>
+          <t>Hosting</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>API Management Consumption</t>
+          <t>Static Web Apps Free</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Monthly included</t>
+          <t>Free tier</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>First 1M API operations/subscription/month</t>
+          <t>Hosting quota shown by the selected plan</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Core shared React SPA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Gateway</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Content Safety F0</t>
+          <t>API Management Consumption</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Free tier</t>
+          <t>Monthly included</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>5,000 text records + 5,000 images/month; hard stop</t>
+          <t>First 1M API operations/subscription/month</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1369,39 +1369,39 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Registry</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Container Registry Standard</t>
+          <t>Content Safety F0</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>12 months</t>
+          <t>Free tier</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1 registry; 100 GB; 10 webhooks</t>
+          <t>5,000 text records + 5,000 images/month; hard stop</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Core: exact Standard SKU</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Registry</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Blob Storage Hot LRS</t>
+          <t>Container Registry Standard</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1411,24 +1411,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>5 GB; 20,000 reads; 10,000 writes</t>
+          <t>1 registry; 100 GB; 10 webhooks</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Core: exact Standard SKU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Security</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Key Vault Standard</t>
+          <t>Blob Storage Hot LRS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1438,7 +1438,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>10,000 RSA-2048 key or secret operations</t>
+          <t>5 GB; 20,000 reads; 10,000 writes</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -1450,12 +1450,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Document AI</t>
+          <t>Security</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Document Intelligence S0</t>
+          <t>Key Vault Standard</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1465,34 +1465,34 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>500 pages</t>
+          <t>10,000 RSA-2048 key or secret operations</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Stretch</t>
+          <t>Core</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>NLP</t>
+          <t>Document AI</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Azure Language</t>
+          <t>Document Intelligence S0</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Always</t>
+          <t>12 months</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>5,000 text records</t>
+          <t>500 pages</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -1504,108 +1504,108 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>NLP</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Functions Consumption</t>
+          <t>Azure Language</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Monthly grant</t>
+          <t>Always</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1M executions + 400,000 GB-s</t>
+          <t>5,000 text records</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Stretch ingestion</t>
+          <t>Stretch</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Event Grid</t>
+          <t>Functions Consumption</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Always</t>
+          <t>Monthly grant</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>100,000 operations/month</t>
+          <t>1M executions + 400,000 GB-s</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Stretch Blob trigger</t>
+          <t>Core durable workflow</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Messaging</t>
+          <t>Events</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Service Bus Standard</t>
+          <t>Event Grid</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>12 months</t>
+          <t>Always</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>750 hours + 13M operations</t>
+          <t>100,000 operations/month</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Defer</t>
+          <t>Stretch Blob trigger</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>Messaging</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Cosmos DB free tier</t>
+          <t>Service Bus Standard</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Always</t>
+          <t>12 months</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1,000 RU/s + 25 GB when free tier selected</t>
+          <t>750 hours + 13M operations</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Defer</t>
+          <t>Core async queue</t>
         </is>
       </c>
     </row>
@@ -1617,152 +1617,206 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL Flexible B1ms</t>
+          <t>Cosmos DB free tier</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>12 months</t>
+          <t>Always</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>750 hours + 32 GB data + 32 GB backup</t>
+          <t>1,000 RU/s + 25 GB when free tier selected</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Defer</t>
+          <t>Core status/audit</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Compute</t>
+          <t>Cache</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Eligible Linux/Windows VMs</t>
+          <t>Azure Managed Redis</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>12 months</t>
+          <t>Paid</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>750 hours each for listed B1s/B2pts v2/B2ats v2</t>
+          <t>No verified free-account grant; hourly SKU charge</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Defer</t>
+          <t>One block if estimate fits; local fallback</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>AI platform</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Foundry</t>
+          <t>PostgreSQL Flexible B1ms</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Platform free</t>
+          <t>12 months</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Consumed features bill at their own rates</t>
+          <t>750 hours + 32 GB data + 32 GB backup</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Defer</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Compute</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Foundry/OpenAI inference</t>
+          <t>Eligible Linux/Windows VMs</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Paid</t>
+          <t>12 months</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>No general free-token grant; model/token rates</t>
+          <t>750 hours each for listed B1s/B2pts v2/B2ats v2</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Core: strict limits</t>
+          <t>Defer</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>AI platform</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Foundry</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Platform free</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Consumed features bill at their own rates</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Foundry/OpenAI inference</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>No general free-token grant; model/token rates</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Core: strict limits</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
           <t>Observability</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Azure Monitor / Log Analytics</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Paid ingestion</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Platform metrics/activity logs have free units; log ingestion metered</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Core: sample/cap</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
         <is>
           <t>Important</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Quotas reset monthly and do not roll over. Exact SKU and the subscription's Cost Management &gt; Free services grid are authoritative. PAYG overages bill the card.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Official list</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>https://azure.microsoft.com/en-us/pricing/free-services/</t>
         </is>
@@ -4363,7 +4417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4453,22 +4507,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Key Vault-backed app configuration</t>
+          <t>Shared website: React SPA with Chat, Document Q&amp;A, and Agent pages</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Key Vault + RBAC</t>
+          <t>Azure Static Web Apps</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Day 7</t>
+          <t>Sprint Day A</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>vault may stay (~$0)</t>
+          <t>destroy Sep 27</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -4484,22 +4538,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Full stack on a VM + TLS + CI deploy-on-push</t>
+          <t>Chat FastAPI: Fargate-equivalent service with cache and TLS</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>VM, VNet, NSG, nginx, TLS</t>
+          <t>Container Apps, ACR, Managed Redis, APIM</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Days 9-12</t>
+          <t>Sprint Day A</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>destroy Day 14</t>
+          <t>Redis same-block; rest Sep 27</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -4515,22 +4569,22 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Container Apps: API + scale-to-zero worker</t>
+          <t>Document Q&amp;A FastAPI: cited RAG</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Container Apps, KEDA, Log Analytics</t>
+          <t>Container Apps, Blob, AI Search, Foundry</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Day 17</t>
+          <t>Sprint Day A</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>destroy Day 21</t>
+          <t>destroy Sep 27</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -4546,22 +4600,22 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Managed PostgreSQL wired through Key Vault</t>
+          <t>Approval-gated Agent FastAPI: durable wait, queue, status</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>PostgreSQL Flexible</t>
+          <t>Durable Functions, Service Bus, Cosmos DB</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Day 17</t>
+          <t>Sprint Day B</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>destroy Day 21 (or keep within free tier)</t>
+          <t>destroy Sep 27</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -4577,22 +4631,22 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>WEBSITE: React UI on Azure Static Web Apps</t>
+          <t>Immutable OIDC redeploy and rollback</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Static Web Apps</t>
+          <t>GitHub Actions, ACR, Container Apps</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Day 19</t>
+          <t>Sprint Day B</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>destroy Day 26</t>
+          <t>destroy Sep 27</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -4601,130 +4655,6 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Rollback + blue/green traffic split drill</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Container Apps revisions</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Day 20</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>AKS: 1-node cluster, deploy, destroy same evening</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>AKS, kubectl</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Day 22</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>destroy same night</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Load-tested + monitored deployment with alerts</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>App Insights, Monitor</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Day 24</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>destroy Day 26</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Full CI/CD: PR -&gt; test -&gt; publish -&gt; deploy -&gt; approve -&gt; rollback</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Actions + OIDC</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Day 25</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add beginner Azure GenAI handbook
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="GenAI Sprint" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Free Quotas" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Daily Plan" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Day Cost Plan" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Deployments" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cost Log" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Destroy Ritual" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GenAI Sprint" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Free Quotas" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Daily Plan" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day Cost Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployments" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cost Log" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Destroy Ritual" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -572,7 +572,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1) GENAI_SOLUTION_OVERVIEW.md/html · 2) GENAI_DEPLOYMENT_GUIDE.md/html · 3) LEARNING_JOURNAL.md/html</t>
+          <t>Start: AZURE_GENAI_BEGINNER_HANDBOOK.md/html/docx · 1) solution overview · 2) deployment guide · 3) journal</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add real-time chat learning app
Amp-Thread-ID: https://ampcode.com/threads/T-01a058ed-9faf-73d8-b500-dfd7e90d2438
</commit_message>
<xml_diff>
--- a/docs/Learning_Tracker.xlsx
+++ b/docs/Learning_Tracker.xlsx
@@ -724,11 +724,19 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Local App 1 React/FastAPI contract implemented: MISS→HIT, zero hit tokens, TTL, scoped keys, and 20-request stampede test verified. Shared Azure platform pending.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">

</xml_diff>